<commit_message>
Rename generic Baseline Estimate Label
</commit_message>
<xml_diff>
--- a/sample_data/DEMO_Tender_Comparison_Workbook.xlsx
+++ b/sample_data/DEMO_Tender_Comparison_Workbook.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fictional sample project for ingestion tests and Stage B demo. SUMMARY first metric pair is Costplan; variance = tender − Costplan.</t>
+          <t>Fictional sample project for ingestion tests and Stage B demo. SUMMARY first metric pair is Baseline Estimate; variance = tender − Baseline Estimate.</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Costplan</t>
+          <t>Baseline Estimate</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -1366,7 +1366,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Variance from Costplan</t>
+          <t>Variance from Baseline Estimate</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1399,7 +1399,7 @@
     <row r="1">
       <c r="C1" t="inlineStr">
         <is>
-          <t>Costplan</t>
+          <t>Baseline Estimate</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="1">
       <c r="C1" t="inlineStr">
         <is>
-          <t>Costplan</t>
+          <t>Baseline Estimate</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">

</xml_diff>